<commit_message>
site build 2026-10-08 21:10
</commit_message>
<xml_diff>
--- a/models/sovereigns/South_Africa_Sovereign_Model.xlsx
+++ b/models/sovereigns/South_Africa_Sovereign_Model.xlsx
@@ -652,12 +652,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>SARB MPC Statement</t>
+          <t>BIS monthly policy rate series</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>23-Sep-26</t>
+          <t>08-Oct-26</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
@@ -678,17 +678,17 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>12m forward</t>
+          <t>Sep-26</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>BER surveys, cited in adjudicated document</t>
+          <t>BER 12-month expectation (as cited in the data record; survey not independently sourced)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>23-Sep-26</t>
+          <t>08-Oct-26</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
@@ -714,12 +714,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Stats SA, CPI August 2026</t>
+          <t>Stats SA via IMF data portal</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>23-Sep-26</t>
+          <t>08-Oct-26</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
@@ -753,11 +753,7 @@
           <t>08-Oct-26</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
-        </is>
-      </c>
+      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -849,7 +845,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>National Treasury MTBPS</t>
+          <t>National Treasury (vintage unverified)</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -950,7 +946,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>23-Sep-26</t>
+          <t>08-Oct-26</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
@@ -997,7 +993,7 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>63.5</v>
+        <v>75.95999999999999</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -1006,22 +1002,22 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Sep-26</t>
+          <t>Aug-26</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>SARB</t>
+          <t>IMF International Liquidity</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>23-Sep-26</t>
+          <t>08-Oct-26</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>gross official FX reserves</t>
+          <t>gross incl. gold ($57.96B ex-gold plus $18.0B gold); SARB headline of $63.5B (Sep-26) has an unresolved definition</t>
         </is>
       </c>
     </row>
@@ -1063,12 +1059,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>SARB</t>
+          <t>SARB (tied to the $63.5B headline reserve figure)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>23-Sep-26</t>
+          <t>08-Oct-26</t>
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
@@ -1131,7 +1127,7 @@
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>479.964</v>
+        <v>480</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -1153,11 +1149,7 @@
           <t>08-Oct-26</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
-        </is>
-      </c>
+      <c r="G22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1279,7 +1271,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>BB</t>
+          <t>BB (foreign) / BB+ (local)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1382,11 +1374,17 @@
           <t>nominal_gdp_usd_bn</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n"/>
+      <c r="B2" s="2" t="n">
+        <v>480</v>
+      </c>
       <c r="C2" s="2" t="n"/>
       <c r="D2" s="2" t="n"/>
       <c r="E2" s="2" t="n"/>
-      <c r="F2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>IMF WEO, 08-Oct-26</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1394,11 +1392,17 @@
           <t>real_gdp_growth_pct</t>
         </is>
       </c>
-      <c r="B3" s="2" t="n"/>
+      <c r="B3" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="C3" s="2" t="n"/>
       <c r="D3" s="2" t="n"/>
       <c r="E3" s="2" t="n"/>
-      <c r="F3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>IMF WEO, 08-Oct-26</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">

</xml_diff>

<commit_message>
site build 2026-10-16 16:38
</commit_message>
<xml_diff>
--- a/models/sovereigns/South_Africa_Sovereign_Model.xlsx
+++ b/models/sovereigns/South_Africa_Sovereign_Model.xlsx
@@ -441,7 +441,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>as of 09-Oct-26</t>
+          <t>as of 16-Oct-26</t>
         </is>
       </c>
     </row>
@@ -590,7 +590,7 @@
       <c r="D1" t="inlineStr"/>
       <c r="E1" t="inlineStr">
         <is>
-          <t>built 12-Oct-26 by pipeline/sovereign_model.py from database/sovereigns/south-africa.json</t>
+          <t>built 16-Oct-26 by pipeline/sovereign_model.py from database/sovereigns/south-africa.json</t>
         </is>
       </c>
     </row>
@@ -652,12 +652,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>BIS monthly policy rate series</t>
+          <t>SARB repo rate (Briefly, 24-Sep-26; EWN, 23-Sep-26)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>08-Oct-26</t>
+          <t>24-Sep-26</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
@@ -678,17 +678,17 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Sep-26</t>
+          <t>12m ahead</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>BER 12-month expectation, cited in adjudicated document (survey not independently sourced)</t>
+          <t>BER survey (as cited in the adjudicated document; not independently sourced)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>08-Oct-26</t>
+          <t>16-Oct-26</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
@@ -719,7 +719,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>08-Oct-26</t>
+          <t>16-Oct-26</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
@@ -745,12 +745,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>IMF WEO</t>
+          <t>IMF WEO (official data record database/sovereigns/south-africa.json)</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>08-Oct-26</t>
+          <t>16-Oct-26</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>77.2</v>
+        <v>77</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -788,22 +788,22 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>medium-term peak</t>
+          <t>end-Mar-25</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>National Treasury MTBPS</t>
+          <t>IMF Article IV press release 26/039</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>08-Oct-26</t>
+          <t>10-Feb-26</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>gross debt, upper end of projected peak range 75.5%-77.2% of GDP</t>
+          <t>IMF Article IV figure; Budget 2026 press reports a 78.9% peak in FY25/26 and the repo holds 77.2%, unreconciled</t>
         </is>
       </c>
     </row>
@@ -813,15 +813,29 @@
           <t>primary_balance_pct_gdp</t>
         </is>
       </c>
-      <c r="B9" s="2" t="n"/>
+      <c r="B9" s="2" t="n">
+        <v>1.6</v>
+      </c>
       <c r="C9" t="inlineStr">
         <is>
           <t>% GDP</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>FY26/27 (main budget, Budget 2026)</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Times Live / Business Day on Budget 2026</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>25-Feb-26</t>
+        </is>
+      </c>
       <c r="G9" t="inlineStr"/>
     </row>
     <row r="10">
@@ -831,7 +845,7 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>-3.8</v>
+        <v>-4</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -840,17 +854,17 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>FY26/27</t>
+          <t>FY26/27 (consolidated, Budget 2026)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>National Treasury, cited via previous document as 'MTBPS 2026'/'Jun-26'; vintage unverified</t>
+          <t>Times Live / Business Day on Budget 2026</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>08-Oct-26</t>
+          <t>25-Feb-26</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
@@ -941,12 +955,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>SARB Quarterly Bulletin</t>
+          <t>SARB</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>08-Oct-26</t>
+          <t>16-Oct-26</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
@@ -1007,17 +1021,17 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>IMF International Liquidity</t>
+          <t>IMF international reserves template</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>08-Oct-26</t>
+          <t>16-Oct-26</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>gross incl. gold (ex-gold $57.96B plus gold $18.0B); SARB headline of $63.5B uses an unresolved definition</t>
+          <t>gross incl. gold (ex-gold $57.96B)</t>
         </is>
       </c>
     </row>
@@ -1027,16 +1041,34 @@
           <t>net_reserves_usd_bn</t>
         </is>
       </c>
-      <c r="B17" s="2" t="n"/>
+      <c r="B17" s="2" t="n">
+        <v>74.3</v>
+      </c>
       <c r="C17" t="inlineStr">
         <is>
           <t>USD bn</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Aug-26</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>IMF international reserves template</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>16-Oct-26</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>gross incl. gold, net of one-year drains</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1271,7 +1303,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>BB (foreign currency) / BB+ (local currency)</t>
+          <t>BB (FC) / BB+ (LC)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1311,11 +1343,6 @@
       <c r="A33" t="inlineStr">
         <is>
           <t>IMF</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>None (Article IV)</t>
         </is>
       </c>
     </row>
@@ -1330,7 +1357,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1344,25 +1371,35 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>2026E</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>2027F</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>2028F</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>FY25/26E</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>FY26/27F</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
@@ -1374,13 +1411,15 @@
           <t>nominal_gdp_usd_bn</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n">
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n">
         <v>480</v>
       </c>
-      <c r="C2" s="2" t="n"/>
       <c r="D2" s="2" t="n"/>
       <c r="E2" s="2" t="n"/>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" t="inlineStr">
         <is>
           <t>IMF WEO, 08-Oct-26</t>
         </is>
@@ -1392,15 +1431,17 @@
           <t>real_gdp_growth_pct</t>
         </is>
       </c>
-      <c r="B3" s="2" t="n">
+      <c r="B3" s="2" t="n"/>
+      <c r="C3" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C3" s="2" t="n"/>
       <c r="D3" s="2" t="n"/>
       <c r="E3" s="2" t="n"/>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>IMF WEO, 08-Oct-26</t>
+      <c r="F3" s="2" t="n"/>
+      <c r="G3" s="2" t="n"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>IMF WEO, repo record, 16-Oct-26 (IMF Article IV, 10-Feb-26, has 1.4% for 2026)</t>
         </is>
       </c>
     </row>
@@ -1414,7 +1455,9 @@
       <c r="C4" s="2" t="n"/>
       <c r="D4" s="2" t="n"/>
       <c r="E4" s="2" t="n"/>
-      <c r="F4" t="inlineStr"/>
+      <c r="F4" s="2" t="n"/>
+      <c r="G4" s="2" t="n"/>
+      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1426,7 +1469,9 @@
       <c r="C5" s="2" t="n"/>
       <c r="D5" s="2" t="n"/>
       <c r="E5" s="2" t="n"/>
-      <c r="F5" t="inlineStr"/>
+      <c r="F5" s="2" t="n"/>
+      <c r="G5" s="2" t="n"/>
+      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1438,17 +1483,23 @@
         <v>-4.5</v>
       </c>
       <c r="C6" s="2" t="n">
+        <v>-4</v>
+      </c>
+      <c r="D6" s="2" t="n">
         <v>-3.8</v>
       </c>
-      <c r="D6" s="2" t="n">
+      <c r="E6" s="2" t="n">
+        <v>-3.1</v>
+      </c>
+      <c r="F6" s="2" t="n">
         <v>-4.5</v>
       </c>
-      <c r="E6" s="2" t="n">
+      <c r="G6" s="2" t="n">
         <v>-3.8</v>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>National Treasury MTBPS, 08-Oct-26 (FY25/26 mapped to 2026E, FY26/27 to 2027F; fiscal year Apr-Mar)</t>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Budget 2026 per Times Live / Business Day, 25-Feb-26; consolidated deficit; fiscal years mapped to the starting calendar year (2025 = FY25/26, 2026E = FY26/27, 2028F = FY28/29)</t>
         </is>
       </c>
     </row>
@@ -1458,11 +1509,25 @@
           <t>primary_balance_pct_gdp</t>
         </is>
       </c>
-      <c r="B7" s="2" t="n"/>
-      <c r="C7" s="2" t="n"/>
-      <c r="D7" s="2" t="n"/>
-      <c r="E7" s="2" t="n"/>
-      <c r="F7" t="inlineStr"/>
+      <c r="B7" s="2" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="F7" s="2" t="n"/>
+      <c r="G7" s="2" t="n"/>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Budget 2026 per Times Live / Business Day, 25-Feb-26; main-budget primary surplus; same fiscal-year mapping</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1473,8 +1538,16 @@
       <c r="B8" s="2" t="n"/>
       <c r="C8" s="2" t="n"/>
       <c r="D8" s="2" t="n"/>
-      <c r="E8" s="2" t="n"/>
-      <c r="F8" t="inlineStr"/>
+      <c r="E8" s="2" t="n">
+        <v>76.5</v>
+      </c>
+      <c r="F8" s="2" t="n"/>
+      <c r="G8" s="2" t="n"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Budget 2026 per Times Live / Business Day, 25-Feb-26; FY28/29 value; the FY25/26 peak is unresolved (77.2% vs 78.9%)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1486,7 +1559,9 @@
       <c r="C9" s="2" t="n"/>
       <c r="D9" s="2" t="n"/>
       <c r="E9" s="2" t="n"/>
-      <c r="F9" t="inlineStr"/>
+      <c r="F9" s="2" t="n"/>
+      <c r="G9" s="2" t="n"/>
+      <c r="H9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1498,7 +1573,9 @@
       <c r="C10" s="2" t="n"/>
       <c r="D10" s="2" t="n"/>
       <c r="E10" s="2" t="n"/>
-      <c r="F10" t="inlineStr"/>
+      <c r="F10" s="2" t="n"/>
+      <c r="G10" s="2" t="n"/>
+      <c r="H10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1510,7 +1587,9 @@
       <c r="C11" s="2" t="n"/>
       <c r="D11" s="2" t="n"/>
       <c r="E11" s="2" t="n"/>
-      <c r="F11" t="inlineStr"/>
+      <c r="F11" s="2" t="n"/>
+      <c r="G11" s="2" t="n"/>
+      <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1522,7 +1601,9 @@
       <c r="C12" s="2" t="n"/>
       <c r="D12" s="2" t="n"/>
       <c r="E12" s="2" t="n"/>
-      <c r="F12" t="inlineStr"/>
+      <c r="F12" s="2" t="n"/>
+      <c r="G12" s="2" t="n"/>
+      <c r="H12" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
site build 2026-10-26 12:05
</commit_message>
<xml_diff>
--- a/models/sovereigns/South_Africa_Sovereign_Model.xlsx
+++ b/models/sovereigns/South_Africa_Sovereign_Model.xlsx
@@ -441,7 +441,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>as of 16-Oct-26</t>
+          <t>as of 26-Oct-26</t>
         </is>
       </c>
     </row>
@@ -652,7 +652,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>SARB repo rate (Briefly, 24-Sep-26; EWN, 23-Sep-26)</t>
+          <t>SARB MPC via EWN and Briefly</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -700,7 +700,7 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>4.4</v>
+        <v>4.5</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -709,17 +709,17 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Aug-26</t>
+          <t>Sep-26</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Stats SA via IMF data portal</t>
+          <t>SAnews (Stats SA); IMF series 4.5455</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>16-Oct-26</t>
+          <t>30-Sep-26</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
@@ -731,7 +731,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -740,17 +740,17 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026E</t>
+          <t>2026F</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>IMF WEO (official data record database/sovereigns/south-africa.json)</t>
+          <t>National Treasury MTBPS via IOL</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>16-Oct-26</t>
+          <t>21-Oct-26</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>77</v>
+        <v>78.2</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -788,22 +788,22 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>end-Mar-25</t>
+          <t>FY26/27</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>IMF Article IV press release 26/039</t>
+          <t>National Treasury MTBPS via IOL and EWN (press summaries)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>10-Feb-26</t>
+          <t>21-Oct-26</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>IMF Article IV figure; Budget 2026 press reports a 78.9% peak in FY25/26 and the repo holds 77.2%, unreconciled</t>
+          <t>gross government debt, FY26/27 (MTBPS); peak 78.4% in FY25/26</t>
         </is>
       </c>
     </row>
@@ -814,7 +814,7 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>1.6</v>
+        <v>1.7</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -823,17 +823,17 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>FY26/27 (main budget, Budget 2026)</t>
+          <t>FY26/27</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Times Live / Business Day on Budget 2026</t>
+          <t>National Treasury MTBPS via IOL</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>25-Feb-26</t>
+          <t>21-Oct-26</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>-4</v>
+        <v>-3.9</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -854,17 +854,17 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>FY26/27 (consolidated, Budget 2026)</t>
+          <t>FY26/27</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Times Live / Business Day on Budget 2026</t>
+          <t>National Treasury MTBPS via IOL and EWN (press summaries)</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>25-Feb-26</t>
+          <t>21-Oct-26</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
@@ -893,7 +893,7 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -902,17 +902,17 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>FY25/26 (floor value, at least 20%)</t>
+          <t>FY25/26</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>National Treasury, cited in the adjudicated document</t>
+          <t>Times Live (debt service R420.6bn)</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>08-Oct-26</t>
+          <t>17-Oct-26</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
@@ -950,7 +950,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Sep-26</t>
+          <t>Sep-26 (four quarters)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -960,7 +960,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>16-Oct-26</t>
+          <t>30-Sep-26</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
@@ -1007,7 +1007,7 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>75.95999999999999</v>
+        <v>75.48</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -1016,22 +1016,22 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Aug-26</t>
+          <t>Sep-26</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>IMF international reserves template</t>
+          <t>IMF</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>16-Oct-26</t>
+          <t>30-Sep-26</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>gross incl. gold (ex-gold $57.96B)</t>
+          <t>gross incl. gold (IMF series); SARB headline of $63.5B (5.8 months of import cover) is not reconciled</t>
         </is>
       </c>
     </row>
@@ -1056,17 +1056,17 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>IMF international reserves template</t>
+          <t>IMF</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>16-Oct-26</t>
+          <t>31-Aug-26</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>gross incl. gold, net of one-year drains</t>
+          <t>gross incl. gold net of one-year drains (IMF reserve template); $58.58B ex-gold at Sep-26</t>
         </is>
       </c>
     </row>
@@ -1335,7 +1335,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>May-26</t>
+          <t>22-May-26</t>
         </is>
       </c>
     </row>
@@ -1357,7 +1357,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1381,25 +1381,35 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>2026F</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>2027F</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>2028F</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>2029F</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>FY25/26E</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>FY26/27F</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
@@ -1419,7 +1429,9 @@
       <c r="E2" s="2" t="n"/>
       <c r="F2" s="2" t="n"/>
       <c r="G2" s="2" t="n"/>
-      <c r="H2" t="inlineStr">
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" t="inlineStr">
         <is>
           <t>IMF WEO, 08-Oct-26</t>
         </is>
@@ -1435,13 +1447,19 @@
       <c r="C3" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D3" s="2" t="n"/>
-      <c r="E3" s="2" t="n"/>
+      <c r="D3" s="2" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>1.6</v>
+      </c>
       <c r="F3" s="2" t="n"/>
       <c r="G3" s="2" t="n"/>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>IMF WEO, repo record, 16-Oct-26 (IMF Article IV, 10-Feb-26, has 1.4% for 2026)</t>
+      <c r="H3" s="2" t="n"/>
+      <c r="I3" s="2" t="n"/>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>National Treasury MTBPS via IOL, 21-Oct-26 (calendar-year forecasts)</t>
         </is>
       </c>
     </row>
@@ -1457,7 +1475,9 @@
       <c r="E4" s="2" t="n"/>
       <c r="F4" s="2" t="n"/>
       <c r="G4" s="2" t="n"/>
-      <c r="H4" t="inlineStr"/>
+      <c r="H4" s="2" t="n"/>
+      <c r="I4" s="2" t="n"/>
+      <c r="J4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1471,7 +1491,9 @@
       <c r="E5" s="2" t="n"/>
       <c r="F5" s="2" t="n"/>
       <c r="G5" s="2" t="n"/>
-      <c r="H5" t="inlineStr"/>
+      <c r="H5" s="2" t="n"/>
+      <c r="I5" s="2" t="n"/>
+      <c r="J5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1483,23 +1505,27 @@
         <v>-4.5</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>-4</v>
-      </c>
-      <c r="D6" s="2" t="n">
+        <v>-3.9</v>
+      </c>
+      <c r="D6" s="2" t="n"/>
+      <c r="E6" s="2" t="n">
         <v>-3.8</v>
       </c>
-      <c r="E6" s="2" t="n">
+      <c r="F6" s="2" t="n">
         <v>-3.1</v>
       </c>
-      <c r="F6" s="2" t="n">
+      <c r="G6" s="2" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="H6" s="2" t="n">
         <v>-4.5</v>
       </c>
-      <c r="G6" s="2" t="n">
+      <c r="I6" s="2" t="n">
         <v>-3.8</v>
       </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Budget 2026 per Times Live / Business Day, 25-Feb-26; consolidated deficit; fiscal years mapped to the starting calendar year (2025 = FY25/26, 2026E = FY26/27, 2028F = FY28/29)</t>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>National Treasury MTBPS via IOL and EWN, 21-Oct-26; fiscal years labelled by start year (2026E = FY26/27, 2029F = FY29/30)</t>
         </is>
       </c>
     </row>
@@ -1513,19 +1539,21 @@
         <v>0.9</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="D7" s="2" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="D7" s="2" t="n"/>
+      <c r="E7" s="2" t="n">
         <v>1.9</v>
       </c>
-      <c r="E7" s="2" t="n">
+      <c r="F7" s="2" t="n">
         <v>2.3</v>
       </c>
-      <c r="F7" s="2" t="n"/>
       <c r="G7" s="2" t="n"/>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Budget 2026 per Times Live / Business Day, 25-Feb-26; main-budget primary surplus; same fiscal-year mapping</t>
+      <c r="H7" s="2" t="n"/>
+      <c r="I7" s="2" t="n"/>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>National Treasury MTBPS via IOL, 21-Oct-26; 2026E = FY26/27</t>
         </is>
       </c>
     </row>
@@ -1535,17 +1563,25 @@
           <t>gov_debt_pct_gdp</t>
         </is>
       </c>
-      <c r="B8" s="2" t="n"/>
-      <c r="C8" s="2" t="n"/>
+      <c r="B8" s="2" t="n">
+        <v>78.40000000000001</v>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>78.2</v>
+      </c>
       <c r="D8" s="2" t="n"/>
-      <c r="E8" s="2" t="n">
+      <c r="E8" s="2" t="n"/>
+      <c r="F8" s="2" t="n">
         <v>76.5</v>
       </c>
-      <c r="F8" s="2" t="n"/>
-      <c r="G8" s="2" t="n"/>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Budget 2026 per Times Live / Business Day, 25-Feb-26; FY28/29 value; the FY25/26 peak is unresolved (77.2% vs 78.9%)</t>
+      <c r="G8" s="2" t="n">
+        <v>76.59999999999999</v>
+      </c>
+      <c r="H8" s="2" t="n"/>
+      <c r="I8" s="2" t="n"/>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>National Treasury MTBPS via IOL and EWN, 21-Oct-26; fiscal years labelled by start year (2025 = FY25/26, 2026E = FY26/27, 2029F = FY29/30)</t>
         </is>
       </c>
     </row>
@@ -1561,7 +1597,9 @@
       <c r="E9" s="2" t="n"/>
       <c r="F9" s="2" t="n"/>
       <c r="G9" s="2" t="n"/>
-      <c r="H9" t="inlineStr"/>
+      <c r="H9" s="2" t="n"/>
+      <c r="I9" s="2" t="n"/>
+      <c r="J9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1575,7 +1613,9 @@
       <c r="E10" s="2" t="n"/>
       <c r="F10" s="2" t="n"/>
       <c r="G10" s="2" t="n"/>
-      <c r="H10" t="inlineStr"/>
+      <c r="H10" s="2" t="n"/>
+      <c r="I10" s="2" t="n"/>
+      <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1589,7 +1629,9 @@
       <c r="E11" s="2" t="n"/>
       <c r="F11" s="2" t="n"/>
       <c r="G11" s="2" t="n"/>
-      <c r="H11" t="inlineStr"/>
+      <c r="H11" s="2" t="n"/>
+      <c r="I11" s="2" t="n"/>
+      <c r="J11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1597,13 +1639,21 @@
           <t>interest_pct_revenue</t>
         </is>
       </c>
-      <c r="B12" s="2" t="n"/>
+      <c r="B12" s="2" t="n">
+        <v>21</v>
+      </c>
       <c r="C12" s="2" t="n"/>
       <c r="D12" s="2" t="n"/>
       <c r="E12" s="2" t="n"/>
       <c r="F12" s="2" t="n"/>
       <c r="G12" s="2" t="n"/>
-      <c r="H12" t="inlineStr"/>
+      <c r="H12" s="2" t="n"/>
+      <c r="I12" s="2" t="n"/>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Times Live, 17-Oct-26; 2025 = FY25/26</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>